<commit_message>
Updated Model with Perfboard
</commit_message>
<xml_diff>
--- a/component-orders.xlsx
+++ b/component-orders.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\projects\primary\auto-water-distribution-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF40C259-EFDD-4454-B5B2-2377D73BBD64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25F98EDB-42C1-4D56-9B26-DACDB41CD174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{38EBA7E1-48E4-4552-B242-4B8FFED322BD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="51">
   <si>
     <t>Name</t>
   </si>
@@ -83,9 +83,6 @@
     <t>JST-PH 2P / 5P</t>
   </si>
   <si>
-    <t>ESP32-DevKitC</t>
-  </si>
-  <si>
     <t>ESP32</t>
   </si>
   <si>
@@ -131,9 +128,6 @@
     <t>AM2302 / DHT22</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>Dip Switch</t>
   </si>
   <si>
@@ -176,10 +170,25 @@
     <t>Perf Board</t>
   </si>
   <si>
-    <t>Screws</t>
-  </si>
-  <si>
     <t>Component Orders</t>
+  </si>
+  <si>
+    <t>Single Sided: 71x51x1</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>ESP32-DevKitC-v4</t>
+  </si>
+  <si>
+    <t>3 - 4</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Bend Pins Flat (Like SMT)</t>
   </si>
 </sst>
 </file>
@@ -252,7 +261,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -287,16 +296,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -306,7 +309,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="22">
     <dxf>
       <font>
         <b val="0"/>
@@ -327,33 +330,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="34" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -377,6 +358,13 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="34" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -399,6 +387,9 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -419,6 +410,9 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -441,6 +435,21 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -482,8 +491,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7503711C-AF0B-4EC7-A40E-90D66D92E0A9}" name="Table13" displayName="Table13" ref="A3:J22" totalsRowCount="1" headerRowDxfId="19" dataDxfId="18">
-  <autoFilter ref="A3:J21" xr:uid="{E7F31172-D701-43B3-B363-E7128DEE1A5A}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7503711C-AF0B-4EC7-A40E-90D66D92E0A9}" name="Table13" displayName="Table13" ref="A3:K21" totalsRowCount="1" headerRowDxfId="21" dataDxfId="20">
+  <autoFilter ref="A3:K20" xr:uid="{E7F31172-D701-43B3-B363-E7128DEE1A5A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -494,21 +503,23 @@
     <filterColumn colId="7" hiddenButton="1"/>
     <filterColumn colId="8" hiddenButton="1"/>
     <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{30505AB0-FB3D-461C-9C3B-2F87CB75CA3E}" name="Name" totalsRowLabel="Total" dataDxfId="17" totalsRowDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{B207E827-F951-4957-A3CD-3D5745D7DBB3}" name="Part Number" dataDxfId="16" totalsRowDxfId="7"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{30505AB0-FB3D-461C-9C3B-2F87CB75CA3E}" name="Name" totalsRowLabel="Total" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{B207E827-F951-4957-A3CD-3D5745D7DBB3}" name="Part Number" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{CF594871-74F7-4898-9EF1-85312228BC79}" name="Notes" dataDxfId="15" totalsRowDxfId="14"/>
     <tableColumn id="5" xr3:uid="{C62F42C1-483F-4CB2-8088-D2891748CED7}" name="Quantity"/>
-    <tableColumn id="7" xr3:uid="{86C5FFE5-26FE-411E-8233-67C26E18EE7D}" name="Price" dataDxfId="15" totalsRowDxfId="6" dataCellStyle="Currency"/>
-    <tableColumn id="11" xr3:uid="{064DACA8-37EA-4944-B852-13399DB8A1F9}" name="Shipping" dataDxfId="14" totalsRowDxfId="5" dataCellStyle="Currency"/>
-    <tableColumn id="4" xr3:uid="{4365DA71-7823-4A6D-B79A-89D229D256C1}" name="PC's" dataDxfId="13" totalsRowDxfId="4" dataCellStyle="Currency"/>
-    <tableColumn id="2" xr3:uid="{B548B73F-E023-486A-8F5B-889414C5F054}" name="Needed to Buy" dataDxfId="12" totalsRowDxfId="3" dataCellStyle="Comma"/>
-    <tableColumn id="8" xr3:uid="{609284FB-B55C-4DDE-B373-81C54EBF78C3}" name="Total Price" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="2" dataCellStyle="Currency">
+    <tableColumn id="7" xr3:uid="{86C5FFE5-26FE-411E-8233-67C26E18EE7D}" name="Price" dataDxfId="13" totalsRowDxfId="12" dataCellStyle="Currency"/>
+    <tableColumn id="11" xr3:uid="{064DACA8-37EA-4944-B852-13399DB8A1F9}" name="Shipping" dataDxfId="11" totalsRowDxfId="10" dataCellStyle="Currency"/>
+    <tableColumn id="4" xr3:uid="{4365DA71-7823-4A6D-B79A-89D229D256C1}" name="PC's" dataDxfId="9" totalsRowDxfId="8" dataCellStyle="Currency"/>
+    <tableColumn id="2" xr3:uid="{B548B73F-E023-486A-8F5B-889414C5F054}" name="Needed to Buy" dataDxfId="7" totalsRowDxfId="6" dataCellStyle="Comma"/>
+    <tableColumn id="8" xr3:uid="{609284FB-B55C-4DDE-B373-81C54EBF78C3}" name="Total Price" totalsRowFunction="custom" dataDxfId="5" totalsRowDxfId="4" dataCellStyle="Currency">
       <calculatedColumnFormula>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</calculatedColumnFormula>
       <totalsRowFormula>SUM(Table13[Total Price])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A5D4A489-4B20-45A7-809F-BD9BDF6944EA}" name="Shipping Time (Days)" dataDxfId="10" totalsRowDxfId="1" dataCellStyle="Currency"/>
-    <tableColumn id="10" xr3:uid="{74DC62F8-6FF4-4011-864C-618358397507}" name="Link" dataDxfId="9" totalsRowDxfId="0" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{A5D4A489-4B20-45A7-809F-BD9BDF6944EA}" name="Shipping Time (Days)" dataDxfId="3" totalsRowDxfId="2" dataCellStyle="Currency"/>
+    <tableColumn id="10" xr3:uid="{74DC62F8-6FF4-4011-864C-618358397507}" name="Link" dataDxfId="1" totalsRowDxfId="0" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="1"/>
 </table>
@@ -831,584 +842,610 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8CFA2BC-95D1-4BFC-A97F-478F653543E5}">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr defaultColWidth="20.7109375" defaultRowHeight="24.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="20.7109375" style="3"/>
+    <col min="1" max="2" width="20.7109375" style="3"/>
+    <col min="3" max="3" width="25.7109375" style="3" customWidth="1"/>
+    <col min="4" max="16384" width="20.7109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:12" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="3"/>
+    </row>
+    <row r="2" spans="1:12" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="3"/>
+    </row>
+    <row r="3" spans="1:12" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L3" s="3"/>
+    </row>
+    <row r="4" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="3"/>
-    </row>
-    <row r="2" spans="1:11" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
-      <c r="D4" s="6">
-        <v>11.29</v>
+      <c r="D4" s="1">
+        <v>1</v>
       </c>
       <c r="E4" s="6">
-        <v>0</v>
-      </c>
-      <c r="F4" s="10">
-        <v>2</v>
-      </c>
-      <c r="G4" s="9">
-        <v>1</v>
-      </c>
-      <c r="H4" s="6">
+        <v>5.95</v>
+      </c>
+      <c r="F4" s="6">
+        <v>0</v>
+      </c>
+      <c r="G4" s="10">
+        <v>1</v>
+      </c>
+      <c r="H4" s="9">
+        <v>1</v>
+      </c>
+      <c r="I4" s="6">
         <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
-        <v>11.29</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.95</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="6">
+      <c r="D5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="6">
         <v>9.99</v>
       </c>
-      <c r="E5" s="6">
-        <v>0</v>
-      </c>
-      <c r="F5" s="10">
+      <c r="F5" s="6">
+        <v>0</v>
+      </c>
+      <c r="G5" s="10">
         <v>420</v>
       </c>
-      <c r="G5" s="9">
-        <v>1</v>
-      </c>
-      <c r="H5" s="6">
+      <c r="H5" s="9">
+        <v>1</v>
+      </c>
+      <c r="I5" s="6">
         <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
         <v>9.99</v>
       </c>
-      <c r="I5" s="11">
-        <v>1</v>
-      </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="11">
+        <v>1</v>
+      </c>
+      <c r="K5" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="1">
-        <v>1</v>
-      </c>
-      <c r="D6" s="6">
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="6">
         <v>2.99</v>
       </c>
-      <c r="E6" s="6">
-        <v>0</v>
-      </c>
-      <c r="F6" s="10">
+      <c r="F6" s="6">
+        <v>0</v>
+      </c>
+      <c r="G6" s="10">
         <v>5</v>
       </c>
-      <c r="G6" s="9">
-        <v>1</v>
-      </c>
-      <c r="H6" s="6">
+      <c r="H6" s="9">
+        <v>1</v>
+      </c>
+      <c r="I6" s="6">
         <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
         <v>2.99</v>
       </c>
-      <c r="I6" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J6" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6">
+        <v>29</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1</v>
+      </c>
+      <c r="E7" s="6">
         <v>3.39</v>
       </c>
-      <c r="E7" s="6">
-        <v>0</v>
-      </c>
-      <c r="F7" s="10">
-        <v>1</v>
-      </c>
-      <c r="G7" s="9">
-        <v>1</v>
-      </c>
-      <c r="H7" s="6">
+      <c r="F7" s="6">
+        <v>0</v>
+      </c>
+      <c r="G7" s="10">
+        <v>1</v>
+      </c>
+      <c r="H7" s="9">
+        <v>1</v>
+      </c>
+      <c r="I7" s="6">
         <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
         <v>3.39</v>
       </c>
-      <c r="I7" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J7" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="1">
         <v>5</v>
       </c>
-      <c r="D8" s="6">
+      <c r="E8" s="6">
         <v>4.62</v>
       </c>
-      <c r="E8" s="6">
+      <c r="F8" s="6">
         <v>1.03</v>
       </c>
-      <c r="F8" s="10">
+      <c r="G8" s="10">
         <v>5</v>
       </c>
-      <c r="G8" s="9">
-        <v>1</v>
-      </c>
-      <c r="H8" s="6">
+      <c r="H8" s="9">
+        <v>1</v>
+      </c>
+      <c r="I8" s="6">
         <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
         <v>5.65</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="J8" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="J8" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="1">
+      <c r="D9" s="1">
         <v>5</v>
       </c>
-      <c r="D9" s="6">
+      <c r="E9" s="6">
         <v>2.86</v>
       </c>
-      <c r="E9" s="6">
-        <v>0</v>
-      </c>
-      <c r="F9" s="10">
+      <c r="F9" s="6">
+        <v>0</v>
+      </c>
+      <c r="G9" s="10">
         <v>10</v>
       </c>
-      <c r="G9" s="9">
-        <v>1</v>
-      </c>
-      <c r="H9" s="13">
+      <c r="H9" s="9">
+        <v>1</v>
+      </c>
+      <c r="I9" s="6">
         <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
         <v>2.86</v>
       </c>
-      <c r="I9" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J9" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="1">
+      <c r="D10" s="1">
         <v>2</v>
       </c>
-      <c r="D10" s="6">
+      <c r="E10" s="6">
         <v>4.99</v>
       </c>
-      <c r="E10" s="6">
-        <v>0</v>
-      </c>
-      <c r="F10" s="10">
+      <c r="F10" s="6">
+        <v>0</v>
+      </c>
+      <c r="G10" s="10">
         <v>20</v>
       </c>
-      <c r="G10" s="9">
-        <v>1</v>
-      </c>
-      <c r="H10" s="13">
+      <c r="H10" s="9">
+        <v>1</v>
+      </c>
+      <c r="I10" s="6">
         <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
         <v>4.99</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="J10" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="J10" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>35</v>
-      </c>
       <c r="B11" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="1">
+        <v>34</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1">
         <v>2</v>
       </c>
-      <c r="D11" s="6">
+      <c r="E11" s="6">
         <v>7.29</v>
       </c>
-      <c r="E11" s="6">
-        <v>0</v>
-      </c>
-      <c r="F11" s="10">
-        <v>1</v>
-      </c>
-      <c r="G11" s="9">
+      <c r="F11" s="6">
+        <v>0</v>
+      </c>
+      <c r="G11" s="10">
+        <v>1</v>
+      </c>
+      <c r="H11" s="9">
         <v>2</v>
       </c>
-      <c r="H11" s="6">
+      <c r="I11" s="6">
         <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
         <v>14.58</v>
       </c>
-      <c r="I11" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J11" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="1">
-        <v>1</v>
-      </c>
-      <c r="D12" s="6">
+        <v>34</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1">
+        <v>1</v>
+      </c>
+      <c r="E12" s="6">
         <v>6.35</v>
       </c>
-      <c r="E12" s="6">
-        <v>0</v>
-      </c>
-      <c r="F12" s="10">
-        <v>1</v>
-      </c>
-      <c r="G12" s="9">
-        <v>1</v>
-      </c>
-      <c r="H12" s="7">
+      <c r="F12" s="6">
+        <v>0</v>
+      </c>
+      <c r="G12" s="10">
+        <v>1</v>
+      </c>
+      <c r="H12" s="9">
+        <v>1</v>
+      </c>
+      <c r="I12" s="7">
         <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
         <v>6.35</v>
       </c>
-      <c r="I12" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J12" s="4" t="s">
+      <c r="J12" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1">
+        <v>6</v>
+      </c>
+      <c r="E13" s="6">
+        <v>0</v>
+      </c>
+      <c r="F13" s="6">
+        <v>0</v>
+      </c>
+      <c r="G13" s="10"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="7">
+        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="11"/>
+      <c r="K13" s="12"/>
+    </row>
+    <row r="14" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="4"/>
+    </row>
+    <row r="15" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="1">
+        <v>3</v>
+      </c>
+      <c r="E15" s="6">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6">
+        <v>0</v>
+      </c>
+      <c r="G15" s="10"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="7">
+        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="1">
+        <v>4</v>
+      </c>
+      <c r="E16" s="6">
+        <v>3.85</v>
+      </c>
+      <c r="F16" s="6">
+        <v>0</v>
+      </c>
+      <c r="G16" s="10">
+        <v>10</v>
+      </c>
+      <c r="H16" s="9">
+        <v>1</v>
+      </c>
+      <c r="I16" s="7">
+        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
+        <v>3.85</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="4"/>
+    </row>
+    <row r="18" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="6">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6">
+        <v>0</v>
+      </c>
+      <c r="G18" s="10"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="7">
+        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="11"/>
+      <c r="K18" s="4"/>
+    </row>
+    <row r="19" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="1">
+      <c r="B19" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="6">
+        <v>0</v>
+      </c>
+      <c r="F19" s="6">
+        <v>0</v>
+      </c>
+      <c r="G19" s="10"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="7">
+        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="11"/>
+      <c r="K19" s="4"/>
+    </row>
+    <row r="20" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="6">
+        <v>0</v>
+      </c>
+      <c r="F20" s="6">
+        <v>0</v>
+      </c>
+      <c r="G20" s="10"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="7">
+        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="11"/>
+      <c r="K20" s="4"/>
+    </row>
+    <row r="21" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="6">
-        <v>0</v>
-      </c>
-      <c r="E13" s="6">
-        <v>0</v>
-      </c>
-      <c r="F13" s="10"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="14">
-        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
-        <v>0</v>
-      </c>
-      <c r="I13" s="11"/>
-      <c r="J13" s="15"/>
-    </row>
-    <row r="14" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="4"/>
-    </row>
-    <row r="15" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="6">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6">
-        <v>0</v>
-      </c>
-      <c r="F15" s="10"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="14">
-        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="11"/>
-      <c r="J15" s="4"/>
-    </row>
-    <row r="16" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="6">
-        <v>0</v>
-      </c>
-      <c r="E16" s="6">
-        <v>0</v>
-      </c>
-      <c r="F16" s="10"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="14">
-        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
-        <v>0</v>
-      </c>
-      <c r="I16" s="11"/>
-      <c r="J16" s="4"/>
-    </row>
-    <row r="17" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="6">
-        <v>0</v>
-      </c>
-      <c r="E17" s="6">
-        <v>0</v>
-      </c>
-      <c r="F17" s="10"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="14">
-        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
-        <v>0</v>
-      </c>
-      <c r="I17" s="11"/>
-      <c r="J17" s="4"/>
-    </row>
-    <row r="18" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="4"/>
-    </row>
-    <row r="19" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="6">
-        <v>0</v>
-      </c>
-      <c r="E19" s="6">
-        <v>0</v>
-      </c>
-      <c r="F19" s="10"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="14">
-        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
-        <v>0</v>
-      </c>
-      <c r="I19" s="11"/>
-      <c r="J19" s="4"/>
-    </row>
-    <row r="20" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="6">
-        <v>0</v>
-      </c>
-      <c r="E20" s="6">
-        <v>0</v>
-      </c>
-      <c r="F20" s="10"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="14">
-        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="11"/>
-      <c r="J20" s="4"/>
-    </row>
-    <row r="21" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="6">
-        <v>0</v>
-      </c>
-      <c r="E21" s="6">
-        <v>0</v>
-      </c>
-      <c r="F21" s="10"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="14">
-        <f>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</f>
-        <v>0</v>
-      </c>
-      <c r="I21" s="11"/>
-      <c r="J21" s="4"/>
-    </row>
-    <row r="22" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C22"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="8">
+      <c r="D21"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="8">
         <f>SUM(Table13[Total Price])</f>
-        <v>62.09</v>
-      </c>
-      <c r="I22" s="8"/>
-      <c r="J22" s="5"/>
+        <v>60.6</v>
+      </c>
+      <c r="J21" s="8"/>
+      <c r="K21" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:J2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:K2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="J4" r:id="rId1" xr:uid="{F0EC4B40-B7F9-4E7A-9381-4D445791A8F3}"/>
-    <hyperlink ref="J10" r:id="rId2" xr:uid="{C8CF97CE-69FE-4D20-ADE3-87B9F2D4B942}"/>
-    <hyperlink ref="J5" r:id="rId3" xr:uid="{EA26A44A-BABD-44C0-8456-8EEFE8D602C2}"/>
-    <hyperlink ref="J11" r:id="rId4" xr:uid="{61E0F56C-82AA-4047-A8D3-B8CFC352553A}"/>
-    <hyperlink ref="J6" r:id="rId5" xr:uid="{9BA54015-9A07-4A0B-9914-7F162A019A7F}"/>
-    <hyperlink ref="J7" r:id="rId6" xr:uid="{54D65BA1-1066-4EA1-9FDF-9C229F0099D8}"/>
-    <hyperlink ref="J8" r:id="rId7" xr:uid="{CF1FEFE9-21B4-4964-B0FC-D03FA48848D5}"/>
-    <hyperlink ref="J9" r:id="rId8" xr:uid="{0A09FFB2-862F-4D18-9BBD-72ECBDE3AE7C}"/>
-    <hyperlink ref="J12" r:id="rId9" xr:uid="{2C1CC6E2-D753-4ABC-9C31-4483EE61FC7E}"/>
+    <hyperlink ref="K4" r:id="rId1" xr:uid="{F0EC4B40-B7F9-4E7A-9381-4D445791A8F3}"/>
+    <hyperlink ref="K10" r:id="rId2" xr:uid="{C8CF97CE-69FE-4D20-ADE3-87B9F2D4B942}"/>
+    <hyperlink ref="K5" r:id="rId3" xr:uid="{EA26A44A-BABD-44C0-8456-8EEFE8D602C2}"/>
+    <hyperlink ref="K11" r:id="rId4" xr:uid="{61E0F56C-82AA-4047-A8D3-B8CFC352553A}"/>
+    <hyperlink ref="K6" r:id="rId5" xr:uid="{9BA54015-9A07-4A0B-9914-7F162A019A7F}"/>
+    <hyperlink ref="K7" r:id="rId6" xr:uid="{54D65BA1-1066-4EA1-9FDF-9C229F0099D8}"/>
+    <hyperlink ref="K8" r:id="rId7" xr:uid="{CF1FEFE9-21B4-4964-B0FC-D03FA48848D5}"/>
+    <hyperlink ref="K9" r:id="rId8" xr:uid="{0A09FFB2-862F-4D18-9BBD-72ECBDE3AE7C}"/>
+    <hyperlink ref="K12" r:id="rId9" xr:uid="{2C1CC6E2-D753-4ABC-9C31-4483EE61FC7E}"/>
+    <hyperlink ref="K16" r:id="rId10" xr:uid="{AE31F1FD-339E-4C5C-872E-AF3A0FBE3889}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId10"/>
+    <tablePart r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Order List with Separated Components
</commit_message>
<xml_diff>
--- a/component-orders.xlsx
+++ b/component-orders.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\projects\primary\regulated-irrigation-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A132CE-3855-4D1F-B1D7-D9BC84951229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E81FA2A2-DEDA-4512-AE13-DBAB14E1EF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{38EBA7E1-48E4-4552-B242-4B8FFED322BD}"/>
   </bookViews>
   <sheets>
     <sheet name="component-orders" sheetId="4" r:id="rId1"/>
-    <sheet name="component-orders_pre-aliexpress" sheetId="5" r:id="rId2"/>
-    <sheet name="component-orders_old" sheetId="3" r:id="rId3"/>
+    <sheet name="component-store-orders" sheetId="6" r:id="rId2"/>
+    <sheet name="-b-pre-aliexpress" sheetId="5" r:id="rId3"/>
+    <sheet name="-b-old" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="140">
   <si>
     <t>Name</t>
   </si>
@@ -295,13 +296,169 @@
     <t>Casing (Model)</t>
   </si>
   <si>
-    <t>AliExpress Parts</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
     <t>AliExpress</t>
+  </si>
+  <si>
+    <t>8 - 12, 18</t>
+  </si>
+  <si>
+    <t>Store</t>
+  </si>
+  <si>
+    <t>3D Print</t>
+  </si>
+  <si>
+    <t>Store Basket</t>
+  </si>
+  <si>
+    <t>Electronics</t>
+  </si>
+  <si>
+    <t>Components</t>
+  </si>
+  <si>
+    <t>1/2" (OD-16mm)</t>
+  </si>
+  <si>
+    <t>Command Module</t>
+  </si>
+  <si>
+    <t>Switch Module</t>
+  </si>
+  <si>
+    <t>v1.0.0</t>
+  </si>
+  <si>
+    <t>B2P-VH(LF)(SN)</t>
+  </si>
+  <si>
+    <t>SS-12D00-G3</t>
+  </si>
+  <si>
+    <t>B5B-PH-K-S(LF)(SN)</t>
+  </si>
+  <si>
+    <t>IRLZ44N(UMW)</t>
+  </si>
+  <si>
+    <t>SB560_AY_10001</t>
+  </si>
+  <si>
+    <t>74HC595N</t>
+  </si>
+  <si>
+    <t>B2B-PH-K-S(LF)(SN)</t>
+  </si>
+  <si>
+    <t>PM2.54-1X3P-H85</t>
+  </si>
+  <si>
+    <t>JST-PH Male 2pin</t>
+  </si>
+  <si>
+    <t>JST-PH Male 5pin</t>
+  </si>
+  <si>
+    <t>JST-VH Male 2pin</t>
+  </si>
+  <si>
+    <t>Header 3pin</t>
+  </si>
+  <si>
+    <t>Temp Sensor</t>
+  </si>
+  <si>
+    <t>DHT22</t>
+  </si>
+  <si>
+    <t>Pipe: Flexible PVC</t>
+  </si>
+  <si>
+    <t>1m: ID-12mm</t>
+  </si>
+  <si>
+    <t>2m: ID-16mm (1/2")</t>
+  </si>
+  <si>
+    <t>T-Piece</t>
+  </si>
+  <si>
+    <t>Pipe Reducer</t>
+  </si>
+  <si>
+    <t>3.9mm - 12.7mm</t>
+  </si>
+  <si>
+    <t>MT3608</t>
+  </si>
+  <si>
+    <t>2A OUT</t>
+  </si>
+  <si>
+    <t>10cm: Double Ended</t>
+  </si>
+  <si>
+    <t>Wire: JST-VH 2pin</t>
+  </si>
+  <si>
+    <t>Wire: JST-PH 5pin</t>
+  </si>
+  <si>
+    <t>Wire: JST-PH 2pin</t>
+  </si>
+  <si>
+    <t>20cm: Single Ended</t>
+  </si>
+  <si>
+    <t>11.1mm - 15.8mm</t>
+  </si>
+  <si>
+    <t>5W: 12V (3m Lift, 280l/h)</t>
+  </si>
+  <si>
+    <t>FPD-270A</t>
+  </si>
+  <si>
+    <t>12V: G1/2" NC</t>
+  </si>
+  <si>
+    <t>ZS-042</t>
+  </si>
+  <si>
+    <t>4Ah: 3.7V</t>
+  </si>
+  <si>
+    <t>8 - 12</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>3.3V: 5A-12V</t>
+  </si>
+  <si>
+    <t>Mosfet</t>
+  </si>
+  <si>
+    <t>5A</t>
+  </si>
+  <si>
+    <t>Diode</t>
+  </si>
+  <si>
+    <t>8bit</t>
+  </si>
+  <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>2state</t>
+  </si>
+  <si>
+    <t>PM2.54-1*19</t>
+  </si>
+  <si>
+    <t>Header 19pin</t>
   </si>
 </sst>
 </file>
@@ -380,7 +537,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -421,7 +578,13 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -431,7 +594,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="64">
+  <dxfs count="84">
     <dxf>
       <font>
         <b val="0"/>
@@ -492,6 +655,51 @@
         <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
@@ -578,6 +786,9 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -906,6 +1117,80 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -927,6 +1212,28 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -941,8 +1248,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D0F5120E-986D-4067-B0C7-38EE2E0158E2}" name="Table132" displayName="Table132" ref="A3:K13" totalsRowCount="1" headerRowDxfId="63" dataDxfId="62">
-  <autoFilter ref="A3:K12" xr:uid="{E7F31172-D701-43B3-B363-E7128DEE1A5A}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D0F5120E-986D-4067-B0C7-38EE2E0158E2}" name="Table132" displayName="Table132" ref="A3:L37" totalsRowCount="1" headerRowDxfId="83" dataDxfId="82">
+  <autoFilter ref="A3:L36" xr:uid="{E7F31172-D701-43B3-B363-E7128DEE1A5A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -954,29 +1261,62 @@
     <filterColumn colId="8" hiddenButton="1"/>
     <filterColumn colId="9" hiddenButton="1"/>
     <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{9E879416-F40A-4624-9F1D-8E3EA9B26E4F}" name="Name" totalsRowLabel="Total" dataDxfId="19" totalsRowDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{39F367DD-94B8-4C39-8D62-42707C3DCD3F}" name="Part Number" dataDxfId="18" totalsRowDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{D136FD14-5D1F-4B27-8E3A-CEAA15545B54}" name="Info" dataDxfId="17" totalsRowDxfId="7"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{9E879416-F40A-4624-9F1D-8E3EA9B26E4F}" name="Store" totalsRowLabel="Total" dataDxfId="29" totalsRowDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{E5C18827-E5F9-4E36-8E09-A33590D1C7BB}" name="Name" dataDxfId="28" totalsRowDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{39F367DD-94B8-4C39-8D62-42707C3DCD3F}" name="Part Number" dataDxfId="27" totalsRowDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{D136FD14-5D1F-4B27-8E3A-CEAA15545B54}" name="Info" dataDxfId="26" totalsRowDxfId="7"/>
     <tableColumn id="5" xr3:uid="{0BC47891-AA27-4760-A86D-FC5961E3AF50}" name="Min Quantity"/>
-    <tableColumn id="7" xr3:uid="{01B4F257-9F3F-47C8-A0AF-616870AD9765}" name="Unit Price" dataDxfId="16" totalsRowDxfId="6" dataCellStyle="Currency"/>
-    <tableColumn id="11" xr3:uid="{F6A62268-004A-4602-947B-BD1B548BEFEF}" name="Shipping" dataDxfId="15" totalsRowDxfId="5" dataCellStyle="Currency"/>
-    <tableColumn id="4" xr3:uid="{663A3CAC-B93E-4703-8B64-0A0819962437}" name="PC's" dataDxfId="14" totalsRowDxfId="4" dataCellStyle="Currency"/>
-    <tableColumn id="2" xr3:uid="{5806903A-DE05-4384-A312-563786E56C58}" name="Needed to Buy" dataDxfId="13" totalsRowDxfId="3" dataCellStyle="Comma"/>
-    <tableColumn id="8" xr3:uid="{A0B50653-0FB1-4D21-8A20-FAA95A4B1F77}" name="Total Price" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="2" dataCellStyle="Currency">
+    <tableColumn id="7" xr3:uid="{01B4F257-9F3F-47C8-A0AF-616870AD9765}" name="Unit Price" dataDxfId="25" totalsRowDxfId="6" dataCellStyle="Currency"/>
+    <tableColumn id="11" xr3:uid="{F6A62268-004A-4602-947B-BD1B548BEFEF}" name="Shipping" dataDxfId="24" totalsRowDxfId="5" dataCellStyle="Currency"/>
+    <tableColumn id="4" xr3:uid="{663A3CAC-B93E-4703-8B64-0A0819962437}" name="PC's" dataDxfId="23" totalsRowDxfId="4" dataCellStyle="Currency"/>
+    <tableColumn id="2" xr3:uid="{5806903A-DE05-4384-A312-563786E56C58}" name="Needed to Buy" dataDxfId="22" totalsRowDxfId="3" dataCellStyle="Comma"/>
+    <tableColumn id="8" xr3:uid="{A0B50653-0FB1-4D21-8A20-FAA95A4B1F77}" name="Total Price" totalsRowFunction="custom" dataDxfId="21" totalsRowDxfId="2" dataCellStyle="Currency">
       <calculatedColumnFormula>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</calculatedColumnFormula>
       <totalsRowFormula>SUM(Table132[Total Price])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{515CF629-198C-414C-AF72-6CFCAEDCCA71}" name="Shipping Time (Days)" dataDxfId="11" totalsRowDxfId="1" dataCellStyle="Currency"/>
-    <tableColumn id="10" xr3:uid="{68DD17EA-77A6-418D-8EA7-0A1B2711C634}" name="Link" dataDxfId="10" totalsRowDxfId="0" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{515CF629-198C-414C-AF72-6CFCAEDCCA71}" name="Shipping Time (Days)" dataDxfId="20" totalsRowDxfId="1" dataCellStyle="Currency"/>
+    <tableColumn id="10" xr3:uid="{68DD17EA-77A6-418D-8EA7-0A1B2711C634}" name="Link" dataDxfId="19" totalsRowDxfId="0" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00975BCA-8754-49BE-95B9-44AA54A5BC1E}" name="Table1324" displayName="Table1324" ref="A3:K19" totalsRowCount="1" headerRowDxfId="61" dataDxfId="60">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A870F7C7-C273-4F13-85A8-F8896C12C9F4}" name="Table1325" displayName="Table1325" ref="A3:I9" totalsRowCount="1" headerRowDxfId="81" dataDxfId="80">
+  <autoFilter ref="A3:I8" xr:uid="{E7F31172-D701-43B3-B363-E7128DEE1A5A}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{39FC1643-C009-45D0-BEAC-B7631C32DA24}" name="Store Basket" totalsRowLabel="Total" dataDxfId="79" totalsRowDxfId="18"/>
+    <tableColumn id="12" xr3:uid="{E1E8FB97-D6C0-4547-9C66-6B16A1884AD6}" name="Info" dataDxfId="78" totalsRowDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{BAB12CC7-BA69-4AC4-B361-A5D9BE286BC4}" name="Min Quantity"/>
+    <tableColumn id="7" xr3:uid="{C17488F9-BC53-4EF5-9040-A1643599EECE}" name="Unit Price" dataDxfId="77" totalsRowDxfId="16" dataCellStyle="Currency"/>
+    <tableColumn id="11" xr3:uid="{9DBCDFBA-1C9B-4A16-A86E-BF582EEC3A8E}" name="Shipping" dataDxfId="76" totalsRowDxfId="15" dataCellStyle="Currency"/>
+    <tableColumn id="2" xr3:uid="{8C88220A-F43F-466B-B51D-C9AE32690669}" name="Needed to Buy" dataDxfId="75" totalsRowDxfId="14" dataCellStyle="Comma"/>
+    <tableColumn id="8" xr3:uid="{D786A848-60A1-48EE-A476-5E0C9A40C298}" name="Total Price" totalsRowFunction="custom" dataDxfId="74" totalsRowDxfId="13" dataCellStyle="Currency">
+      <calculatedColumnFormula>Table1325[[#This Row],[Unit Price]]*Table1325[[#This Row],[Needed to Buy]]+Table1325[[#This Row],[Shipping]]</calculatedColumnFormula>
+      <totalsRowFormula>SUM(Table1325[Total Price])</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{72B5CE47-971F-4990-87B1-19804E9DE094}" name="Shipping Time (Days)" dataDxfId="73" totalsRowDxfId="12" dataCellStyle="Currency"/>
+    <tableColumn id="10" xr3:uid="{0B2088CA-3B32-4118-8FB4-509134215037}" name="Link" dataDxfId="72" totalsRowDxfId="11" dataCellStyle="Hyperlink"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00975BCA-8754-49BE-95B9-44AA54A5BC1E}" name="Table1324" displayName="Table1324" ref="A3:K19" totalsRowCount="1" headerRowDxfId="71" dataDxfId="70">
   <autoFilter ref="A3:K18" xr:uid="{E7F31172-D701-43B3-B363-E7128DEE1A5A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -991,27 +1331,27 @@
     <filterColumn colId="10" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{C346CA06-C1C4-43A6-8295-62F940DCE5B3}" name="Name" totalsRowLabel="Total" dataDxfId="59" totalsRowDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{BE978B11-205C-4C8B-A924-1483998F3883}" name="Part Number" dataDxfId="57" totalsRowDxfId="56"/>
-    <tableColumn id="12" xr3:uid="{F82F865A-27C9-488A-8535-F250CC5B28B4}" name="Info" dataDxfId="55" totalsRowDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{C346CA06-C1C4-43A6-8295-62F940DCE5B3}" name="Name" totalsRowLabel="Total" dataDxfId="69" totalsRowDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{BE978B11-205C-4C8B-A924-1483998F3883}" name="Part Number" dataDxfId="67" totalsRowDxfId="66"/>
+    <tableColumn id="12" xr3:uid="{F82F865A-27C9-488A-8535-F250CC5B28B4}" name="Info" dataDxfId="65" totalsRowDxfId="64"/>
     <tableColumn id="5" xr3:uid="{F9DD1078-54BD-4F42-9C8E-58C2DD310E53}" name="Min Quantity"/>
-    <tableColumn id="7" xr3:uid="{73DC3B50-2DA1-4C4A-88F3-5058FEBBF6A4}" name="Unit Price" dataDxfId="53" totalsRowDxfId="52" dataCellStyle="Currency"/>
-    <tableColumn id="11" xr3:uid="{8BAB5064-5E4C-48EB-9CA1-D0507D9EA1C0}" name="Shipping" dataDxfId="51" totalsRowDxfId="50" dataCellStyle="Currency"/>
-    <tableColumn id="4" xr3:uid="{2D48F19F-79DE-48E1-A3FC-7BA806532C00}" name="PC's" dataDxfId="49" totalsRowDxfId="48" dataCellStyle="Currency"/>
-    <tableColumn id="2" xr3:uid="{B1CB06A2-3AAF-435A-8624-0A7549DB6267}" name="Needed to Buy" dataDxfId="47" totalsRowDxfId="46" dataCellStyle="Comma"/>
-    <tableColumn id="8" xr3:uid="{EDEA9E1A-C648-4FE2-B8B2-71100366E852}" name="Total Price" totalsRowFunction="custom" dataDxfId="45" totalsRowDxfId="44" dataCellStyle="Currency">
+    <tableColumn id="7" xr3:uid="{73DC3B50-2DA1-4C4A-88F3-5058FEBBF6A4}" name="Unit Price" dataDxfId="63" totalsRowDxfId="62" dataCellStyle="Currency"/>
+    <tableColumn id="11" xr3:uid="{8BAB5064-5E4C-48EB-9CA1-D0507D9EA1C0}" name="Shipping" dataDxfId="61" totalsRowDxfId="60" dataCellStyle="Currency"/>
+    <tableColumn id="4" xr3:uid="{2D48F19F-79DE-48E1-A3FC-7BA806532C00}" name="PC's" dataDxfId="59" totalsRowDxfId="58" dataCellStyle="Currency"/>
+    <tableColumn id="2" xr3:uid="{B1CB06A2-3AAF-435A-8624-0A7549DB6267}" name="Needed to Buy" dataDxfId="57" totalsRowDxfId="56" dataCellStyle="Comma"/>
+    <tableColumn id="8" xr3:uid="{EDEA9E1A-C648-4FE2-B8B2-71100366E852}" name="Total Price" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="54" dataCellStyle="Currency">
       <calculatedColumnFormula>Table1324[[#This Row],[Unit Price]]*Table1324[[#This Row],[Needed to Buy]]+Table1324[[#This Row],[Shipping]]</calculatedColumnFormula>
       <totalsRowFormula>SUM(Table1324[Total Price])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0F38EF4B-9C7E-4E08-8FD9-3A0D5506B851}" name="Shipping Time (Days)" dataDxfId="43" totalsRowDxfId="42" dataCellStyle="Currency"/>
-    <tableColumn id="10" xr3:uid="{CA6C939D-FE5F-4B38-9659-94D7C8EF0A98}" name="Link" dataDxfId="41" totalsRowDxfId="40" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{0F38EF4B-9C7E-4E08-8FD9-3A0D5506B851}" name="Shipping Time (Days)" dataDxfId="53" totalsRowDxfId="52" dataCellStyle="Currency"/>
+    <tableColumn id="10" xr3:uid="{CA6C939D-FE5F-4B38-9659-94D7C8EF0A98}" name="Link" dataDxfId="51" totalsRowDxfId="50" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="1"/>
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7503711C-AF0B-4EC7-A40E-90D66D92E0A9}" name="Table13" displayName="Table13" ref="A3:J21" totalsRowCount="1" headerRowDxfId="39" dataDxfId="38">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7503711C-AF0B-4EC7-A40E-90D66D92E0A9}" name="Table13" displayName="Table13" ref="A3:J21" totalsRowCount="1" headerRowDxfId="49" dataDxfId="48">
   <autoFilter ref="A3:J20" xr:uid="{E7F31172-D701-43B3-B363-E7128DEE1A5A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1025,19 +1365,19 @@
     <filterColumn colId="9" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{30505AB0-FB3D-461C-9C3B-2F87CB75CA3E}" name="Name" totalsRowLabel="Total" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{B207E827-F951-4957-A3CD-3D5745D7DBB3}" name="Part Number" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{30505AB0-FB3D-461C-9C3B-2F87CB75CA3E}" name="Name" totalsRowLabel="Total" dataDxfId="47" totalsRowDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{B207E827-F951-4957-A3CD-3D5745D7DBB3}" name="Part Number" dataDxfId="45" totalsRowDxfId="44"/>
     <tableColumn id="5" xr3:uid="{C62F42C1-483F-4CB2-8088-D2891748CED7}" name="Quantity"/>
-    <tableColumn id="7" xr3:uid="{86C5FFE5-26FE-411E-8233-67C26E18EE7D}" name="Price" dataDxfId="33" totalsRowDxfId="32" dataCellStyle="Currency"/>
-    <tableColumn id="11" xr3:uid="{064DACA8-37EA-4944-B852-13399DB8A1F9}" name="Shipping" dataDxfId="31" totalsRowDxfId="30" dataCellStyle="Currency"/>
-    <tableColumn id="4" xr3:uid="{4365DA71-7823-4A6D-B79A-89D229D256C1}" name="PC's" dataDxfId="29" totalsRowDxfId="28" dataCellStyle="Currency"/>
-    <tableColumn id="2" xr3:uid="{B548B73F-E023-486A-8F5B-889414C5F054}" name="Needed to Buy" dataDxfId="27" totalsRowDxfId="26" dataCellStyle="Comma"/>
-    <tableColumn id="8" xr3:uid="{609284FB-B55C-4DDE-B373-81C54EBF78C3}" name="Total Price" totalsRowFunction="custom" dataDxfId="25" totalsRowDxfId="24" dataCellStyle="Currency">
+    <tableColumn id="7" xr3:uid="{86C5FFE5-26FE-411E-8233-67C26E18EE7D}" name="Price" dataDxfId="43" totalsRowDxfId="42" dataCellStyle="Currency"/>
+    <tableColumn id="11" xr3:uid="{064DACA8-37EA-4944-B852-13399DB8A1F9}" name="Shipping" dataDxfId="41" totalsRowDxfId="40" dataCellStyle="Currency"/>
+    <tableColumn id="4" xr3:uid="{4365DA71-7823-4A6D-B79A-89D229D256C1}" name="PC's" dataDxfId="39" totalsRowDxfId="38" dataCellStyle="Currency"/>
+    <tableColumn id="2" xr3:uid="{B548B73F-E023-486A-8F5B-889414C5F054}" name="Needed to Buy" dataDxfId="37" totalsRowDxfId="36" dataCellStyle="Comma"/>
+    <tableColumn id="8" xr3:uid="{609284FB-B55C-4DDE-B373-81C54EBF78C3}" name="Total Price" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="34" dataCellStyle="Currency">
       <calculatedColumnFormula>Table13[[#This Row],[Price]]*Table13[[#This Row],[Needed to Buy]]+Table13[[#This Row],[Shipping]]</calculatedColumnFormula>
       <totalsRowFormula>SUM(Table13[Total Price])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A5D4A489-4B20-45A7-809F-BD9BDF6944EA}" name="Shipping Time (Days)" dataDxfId="23" totalsRowDxfId="22" dataCellStyle="Currency"/>
-    <tableColumn id="10" xr3:uid="{74DC62F8-6FF4-4011-864C-618358397507}" name="Link" dataDxfId="21" totalsRowDxfId="20" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{A5D4A489-4B20-45A7-809F-BD9BDF6944EA}" name="Shipping Time (Days)" dataDxfId="33" totalsRowDxfId="32" dataCellStyle="Currency"/>
+    <tableColumn id="10" xr3:uid="{74DC62F8-6FF4-4011-864C-618358397507}" name="Link" dataDxfId="31" totalsRowDxfId="30" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="1"/>
 </table>
@@ -1360,414 +1700,1583 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA52A867-AF99-4863-B5FF-AF28D5FD4C20}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr defaultColWidth="20.7109375" defaultRowHeight="24.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="3"/>
-    <col min="2" max="2" width="20.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" style="3" customWidth="1"/>
-    <col min="5" max="6" width="20.7109375" style="3"/>
-    <col min="7" max="8" width="15.7109375" style="3" customWidth="1"/>
-    <col min="9" max="10" width="20.7109375" style="3"/>
-    <col min="11" max="11" width="10.7109375" style="3" customWidth="1"/>
-    <col min="12" max="16384" width="20.7109375" style="3"/>
+    <col min="1" max="2" width="20.7109375" style="3"/>
+    <col min="3" max="3" width="20.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" style="3" customWidth="1"/>
+    <col min="6" max="7" width="20.7109375" style="3"/>
+    <col min="8" max="9" width="15.7109375" style="3" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" style="3"/>
+    <col min="11" max="11" width="20.7109375" style="3" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" style="3" customWidth="1"/>
+    <col min="13" max="16384" width="20.7109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:13" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="3"/>
-    </row>
-    <row r="2" spans="1:12" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="3"/>
+    </row>
+    <row r="2" spans="1:13" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14" t="s">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="3"/>
-    </row>
-    <row r="3" spans="1:12" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="3"/>
+    </row>
+    <row r="3" spans="1:13" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="3"/>
-    </row>
-    <row r="4" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="H4" s="10"/>
+      <c r="I4" s="9">
+        <v>1</v>
+      </c>
+      <c r="J4" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0.86</v>
+      </c>
+      <c r="G5" s="6">
+        <v>0</v>
+      </c>
+      <c r="H5" s="10">
+        <v>5</v>
+      </c>
+      <c r="I5" s="9">
+        <v>1</v>
+      </c>
+      <c r="J5" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.86</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="14"/>
+    </row>
+    <row r="6" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1</v>
+      </c>
+      <c r="F6" s="6">
+        <v>0.86</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0</v>
+      </c>
+      <c r="H6" s="10">
+        <v>5</v>
+      </c>
+      <c r="I6" s="9">
+        <v>1</v>
+      </c>
+      <c r="J6" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.86</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="14"/>
+    </row>
+    <row r="7" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="6">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G7" s="6">
+        <v>5.94</v>
+      </c>
+      <c r="H7" s="10"/>
+      <c r="I7" s="9">
+        <v>1</v>
+      </c>
+      <c r="J7" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>8.14</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="M7" s="1"/>
+    </row>
+    <row r="8" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="1">
+        <v>3</v>
+      </c>
+      <c r="F8" s="6">
+        <v>0.41</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0</v>
+      </c>
+      <c r="H8" s="10">
+        <v>10</v>
+      </c>
+      <c r="I8" s="9">
+        <v>1</v>
+      </c>
+      <c r="J8" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.41</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="M8" s="1"/>
+    </row>
+    <row r="9" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1</v>
+      </c>
+      <c r="F9" s="6">
+        <v>0.16</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="H9" s="10">
+        <v>3</v>
+      </c>
+      <c r="I9" s="9">
+        <v>1</v>
+      </c>
+      <c r="J9" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.16</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="M9" s="1"/>
+    </row>
+    <row r="10" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" s="1">
+        <v>3</v>
+      </c>
+      <c r="F10" s="6">
+        <v>0.38</v>
+      </c>
+      <c r="G10" s="6">
+        <v>0</v>
+      </c>
+      <c r="H10" s="10">
+        <v>10</v>
+      </c>
+      <c r="I10" s="9">
+        <v>1</v>
+      </c>
+      <c r="J10" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.38</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="M10" s="1"/>
+    </row>
+    <row r="11" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E11" s="1">
+        <v>6</v>
+      </c>
+      <c r="F11" s="6">
+        <v>3.22</v>
+      </c>
+      <c r="G11" s="6">
+        <v>0</v>
+      </c>
+      <c r="H11" s="10">
         <v>15</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="I11" s="9">
+        <v>1</v>
+      </c>
+      <c r="J11" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>3.22</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="M11" s="1"/>
+    </row>
+    <row r="12" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E12" s="1">
+        <v>6</v>
+      </c>
+      <c r="F12" s="6">
+        <v>1.34</v>
+      </c>
+      <c r="G12" s="6">
+        <v>0</v>
+      </c>
+      <c r="H12" s="10">
+        <v>15</v>
+      </c>
+      <c r="I12" s="9">
+        <v>1</v>
+      </c>
+      <c r="J12" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>1.34</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="M12" s="1"/>
+    </row>
+    <row r="13" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E13" s="1">
+        <v>1</v>
+      </c>
+      <c r="F13" s="6">
+        <v>0.52</v>
+      </c>
+      <c r="G13" s="6">
+        <v>0</v>
+      </c>
+      <c r="H13" s="10">
+        <v>5</v>
+      </c>
+      <c r="I13" s="9">
+        <v>1</v>
+      </c>
+      <c r="J13" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.52</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L13" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="M13" s="1"/>
+    </row>
+    <row r="14" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0.43</v>
+      </c>
+      <c r="G14" s="6">
+        <v>0</v>
+      </c>
+      <c r="H14" s="10">
+        <v>20</v>
+      </c>
+      <c r="I14" s="9">
+        <v>1</v>
+      </c>
+      <c r="J14" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.43</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="M14" s="1"/>
+    </row>
+    <row r="15" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15" s="6">
+        <v>0.11</v>
+      </c>
+      <c r="G15" s="6">
+        <v>0</v>
+      </c>
+      <c r="H15" s="10">
+        <v>5</v>
+      </c>
+      <c r="I15" s="9">
+        <v>1</v>
+      </c>
+      <c r="J15" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.11</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="M15" s="1"/>
+    </row>
+    <row r="16" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E16" s="1">
+        <v>2</v>
+      </c>
+      <c r="F16" s="6">
+        <v>0.69</v>
+      </c>
+      <c r="G16" s="6">
+        <v>0</v>
+      </c>
+      <c r="H16" s="10">
+        <v>5</v>
+      </c>
+      <c r="I16" s="9">
+        <v>1</v>
+      </c>
+      <c r="J16" s="16">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.69</v>
+      </c>
+      <c r="K16" s="11"/>
+      <c r="L16" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="M16" s="1"/>
+    </row>
+    <row r="17" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" s="1"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="9">
+        <v>1</v>
+      </c>
+      <c r="J17" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1</v>
+      </c>
+      <c r="F18" s="6">
+        <v>1.79</v>
+      </c>
+      <c r="G18" s="6">
+        <v>0</v>
+      </c>
+      <c r="H18" s="10">
+        <v>1</v>
+      </c>
+      <c r="I18" s="9">
+        <v>1</v>
+      </c>
+      <c r="J18" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>1.79</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L18" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E19" s="1">
+        <v>1</v>
+      </c>
+      <c r="F19" s="6">
+        <v>3.09</v>
+      </c>
+      <c r="G19" s="6">
+        <v>0</v>
+      </c>
+      <c r="H19" s="10">
+        <v>1</v>
+      </c>
+      <c r="I19" s="9">
+        <v>1</v>
+      </c>
+      <c r="J19" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>3.09</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L19" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="E20" s="1">
+        <v>2</v>
+      </c>
+      <c r="F20" s="6">
+        <v>0.76</v>
+      </c>
+      <c r="G20" s="6">
+        <v>0</v>
+      </c>
+      <c r="H20" s="10">
+        <v>5</v>
+      </c>
+      <c r="I20" s="9">
+        <v>1</v>
+      </c>
+      <c r="J20" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.76</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L20" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E21" s="1">
+        <v>2</v>
+      </c>
+      <c r="F21" s="6">
+        <v>1.89</v>
+      </c>
+      <c r="G21" s="6">
+        <v>0</v>
+      </c>
+      <c r="H21" s="10">
+        <v>5</v>
+      </c>
+      <c r="I21" s="9">
+        <v>1</v>
+      </c>
+      <c r="J21" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>1.89</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L21" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22" s="1">
+        <v>2</v>
+      </c>
+      <c r="F22" s="6">
+        <v>1.27</v>
+      </c>
+      <c r="G22" s="6">
+        <v>0</v>
+      </c>
+      <c r="H22" s="10">
+        <v>5</v>
+      </c>
+      <c r="I22" s="9">
+        <v>1</v>
+      </c>
+      <c r="J22" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>1.27</v>
+      </c>
+      <c r="K22" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L22" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E23" s="1">
+        <v>1</v>
+      </c>
+      <c r="F23" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="G23" s="6">
+        <v>0</v>
+      </c>
+      <c r="H23" s="10">
+        <v>10</v>
+      </c>
+      <c r="I23" s="9">
+        <v>1</v>
+      </c>
+      <c r="J23" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0.9</v>
+      </c>
+      <c r="K23" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L23" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E24" s="1">
+        <v>2</v>
+      </c>
+      <c r="F24" s="6">
+        <v>1.82</v>
+      </c>
+      <c r="G24" s="6">
+        <v>0</v>
+      </c>
+      <c r="H24" s="10">
+        <v>10</v>
+      </c>
+      <c r="I24" s="9">
+        <v>1</v>
+      </c>
+      <c r="J24" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>1.82</v>
+      </c>
+      <c r="K24" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L24" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E25" s="1">
+        <v>3</v>
+      </c>
+      <c r="F25" s="6">
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="G25" s="6">
+        <v>0</v>
+      </c>
+      <c r="H25" s="10">
+        <v>5</v>
+      </c>
+      <c r="I25" s="9">
+        <v>1</v>
+      </c>
+      <c r="J25" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="K25" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L25" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E26" s="1">
+        <v>1</v>
+      </c>
+      <c r="F26" s="6">
+        <v>3.83</v>
+      </c>
+      <c r="G26" s="6">
+        <v>0</v>
+      </c>
+      <c r="H26" s="10">
+        <v>1</v>
+      </c>
+      <c r="I26" s="9">
+        <v>1</v>
+      </c>
+      <c r="J26" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>3.83</v>
+      </c>
+      <c r="K26" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L26" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E27" s="1">
+        <v>2</v>
+      </c>
+      <c r="F27" s="6">
+        <v>3.08</v>
+      </c>
+      <c r="G27" s="6">
+        <v>0</v>
+      </c>
+      <c r="H27" s="10">
+        <v>1</v>
+      </c>
+      <c r="I27" s="9">
+        <v>2</v>
+      </c>
+      <c r="J27" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>6.16</v>
+      </c>
+      <c r="K27" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L27" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E28" s="1">
+        <v>1</v>
+      </c>
+      <c r="F28" s="6">
+        <v>1.94</v>
+      </c>
+      <c r="G28" s="6">
+        <v>0</v>
+      </c>
+      <c r="H28" s="10">
+        <v>1</v>
+      </c>
+      <c r="I28" s="9">
+        <v>1</v>
+      </c>
+      <c r="J28" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>1.94</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L28" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="3">
+        <v>5050100</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E29" s="1">
+        <v>1</v>
+      </c>
+      <c r="F29" s="6">
+        <v>5.99</v>
+      </c>
+      <c r="G29" s="6">
+        <v>2.81</v>
+      </c>
+      <c r="H29" s="10">
+        <v>1</v>
+      </c>
+      <c r="I29" s="9">
+        <v>1</v>
+      </c>
+      <c r="J29" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="L29" s="14" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E30" s="1"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="9">
+        <v>1</v>
+      </c>
+      <c r="J30" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0</v>
+      </c>
+      <c r="K30" s="11"/>
+      <c r="L30" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="1">
-        <v>1</v>
-      </c>
-      <c r="E4" s="6">
+      <c r="E31" s="1">
+        <v>1</v>
+      </c>
+      <c r="F31" s="6">
         <v>5.95</v>
       </c>
-      <c r="F4" s="6">
-        <v>0</v>
-      </c>
-      <c r="G4" s="10">
-        <v>1</v>
-      </c>
-      <c r="H4" s="9">
-        <v>1</v>
-      </c>
-      <c r="I4" s="6">
+      <c r="G31" s="6">
+        <v>0</v>
+      </c>
+      <c r="H31" s="10">
+        <v>1</v>
+      </c>
+      <c r="I31" s="9">
+        <v>1</v>
+      </c>
+      <c r="J31" s="6">
         <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
         <v>5.95</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="K31" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="L31" s="14" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1">
-        <v>2</v>
-      </c>
-      <c r="E5" s="6">
-        <v>1.72</v>
-      </c>
-      <c r="F5" s="6">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="G5" s="10">
-        <v>10</v>
-      </c>
-      <c r="H5" s="9">
-        <v>1</v>
-      </c>
-      <c r="I5" s="6">
-        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
-        <v>2.84</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="6">
-        <v>6.86</v>
-      </c>
-      <c r="F6" s="6">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="G6" s="10">
-        <v>1</v>
-      </c>
-      <c r="H6" s="9">
-        <v>1</v>
-      </c>
-      <c r="I6" s="6">
-        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
-        <v>11.96</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D7" s="1">
-        <v>8</v>
-      </c>
-      <c r="E7" s="6">
-        <v>30.35</v>
-      </c>
-      <c r="F7" s="6">
-        <v>2.81</v>
-      </c>
-      <c r="G7" s="10">
-        <v>16</v>
-      </c>
-      <c r="H7" s="9">
-        <v>1</v>
-      </c>
-      <c r="I7" s="6">
-        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
-        <v>33.160000000000004</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="32" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D32" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="1">
-        <v>1</v>
-      </c>
-      <c r="E8" s="6">
+      <c r="E32" s="1">
+        <v>1</v>
+      </c>
+      <c r="F32" s="6">
         <v>2.88</v>
       </c>
-      <c r="F8" s="6">
+      <c r="G32" s="6">
         <v>1.66</v>
       </c>
-      <c r="G8" s="10">
-        <v>1</v>
-      </c>
-      <c r="H8" s="9">
-        <v>1</v>
-      </c>
-      <c r="I8" s="6">
+      <c r="H32" s="10">
+        <v>1</v>
+      </c>
+      <c r="I32" s="9">
+        <v>1</v>
+      </c>
+      <c r="J32" s="6">
         <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
         <v>4.54</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="K32" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="L32" s="14" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="33" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D33" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="1">
-        <v>1</v>
-      </c>
-      <c r="E9" s="6">
+      <c r="E33" s="1">
+        <v>1</v>
+      </c>
+      <c r="F33" s="6">
         <v>2.74</v>
       </c>
-      <c r="F9" s="6">
-        <v>0</v>
-      </c>
-      <c r="G9" s="10">
-        <v>1</v>
-      </c>
-      <c r="H9" s="9">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6">
+      <c r="G33" s="6">
+        <v>0</v>
+      </c>
+      <c r="H33" s="10">
+        <v>1</v>
+      </c>
+      <c r="I33" s="9">
+        <v>1</v>
+      </c>
+      <c r="J33" s="6">
         <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
         <v>2.74</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="K33" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="L33" s="14" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="6">
-        <v>0</v>
-      </c>
-      <c r="F10" s="6">
-        <v>0</v>
-      </c>
-      <c r="G10" s="10"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="6">
-        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="11"/>
-      <c r="K10" s="4"/>
-    </row>
-    <row r="11" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D11" s="1">
-        <v>1</v>
-      </c>
-      <c r="E11" s="6">
+    <row r="34" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E34" s="1">
+        <v>1</v>
+      </c>
+      <c r="F34" s="6">
         <v>3.8</v>
       </c>
-      <c r="F11" s="6">
-        <v>0</v>
-      </c>
-      <c r="G11" s="10">
-        <v>1</v>
-      </c>
-      <c r="H11" s="9">
-        <v>1</v>
-      </c>
-      <c r="I11" s="6">
+      <c r="G34" s="6">
+        <v>0</v>
+      </c>
+      <c r="H34" s="10">
+        <v>1</v>
+      </c>
+      <c r="I34" s="9">
+        <v>1</v>
+      </c>
+      <c r="J34" s="6">
         <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
         <v>3.8</v>
       </c>
-      <c r="J11" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="K11" s="4" t="s">
+      <c r="K34" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="L34" s="14" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D12" s="1">
+    <row r="35" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E35" s="1">
         <v>2</v>
       </c>
-      <c r="E12" s="6">
+      <c r="F35" s="6">
         <v>3.99</v>
       </c>
-      <c r="F12" s="6">
-        <v>0</v>
-      </c>
-      <c r="G12" s="10">
-        <v>5</v>
-      </c>
-      <c r="H12" s="9">
-        <v>1</v>
-      </c>
-      <c r="I12" s="6">
+      <c r="G35" s="6">
+        <v>0</v>
+      </c>
+      <c r="H35" s="10">
+        <v>2</v>
+      </c>
+      <c r="I35" s="9">
+        <v>1</v>
+      </c>
+      <c r="J35" s="6">
         <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
         <v>3.99</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="K35" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="L35" s="14" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+    <row r="36" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E36" s="1">
+        <v>1</v>
+      </c>
+      <c r="F36" s="6">
+        <v>0</v>
+      </c>
+      <c r="G36" s="6">
+        <v>0</v>
+      </c>
+      <c r="H36" s="10"/>
+      <c r="I36" s="9">
+        <v>1</v>
+      </c>
+      <c r="J36" s="6">
+        <f>Table132[[#This Row],[Unit Price]]*Table132[[#This Row],[Needed to Buy]]+Table132[[#This Row],[Shipping]]</f>
+        <v>0</v>
+      </c>
+      <c r="K36" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="L36" s="4"/>
+    </row>
+    <row r="37" spans="1:12" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D13"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="8">
+      <c r="E37"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="8">
         <f>SUM(Table132[Total Price])</f>
-        <v>68.98</v>
-      </c>
-      <c r="J13" s="8"/>
-      <c r="K13" s="5"/>
+        <v>73.52</v>
+      </c>
+      <c r="K37" s="8"/>
+      <c r="L37" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:K2"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:L2"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="K4" r:id="rId1" xr:uid="{4DDFA626-C1E3-4458-92A2-B7D165A0519C}"/>
-    <hyperlink ref="K5" r:id="rId2" xr:uid="{FB6AA4AF-9C94-4435-9586-AF25E82C1959}"/>
-    <hyperlink ref="K6" r:id="rId3" xr:uid="{5ABDACB3-B3F4-4F86-99EC-4AA62FA84D21}"/>
-    <hyperlink ref="K7" r:id="rId4" xr:uid="{6459CE0B-A281-4375-9C7C-05121ADE6BE2}"/>
-    <hyperlink ref="K8" r:id="rId5" xr:uid="{018F4AFE-A58A-48E7-A5D8-D49BBBA7AF38}"/>
-    <hyperlink ref="K9" r:id="rId6" xr:uid="{84533807-29E2-4CAA-84C9-34900C15055C}"/>
-    <hyperlink ref="K12" r:id="rId7" xr:uid="{C14D6FD1-AEE2-4ECD-A527-6196769534BB}"/>
-    <hyperlink ref="K11" r:id="rId8" xr:uid="{1D36EC75-443F-4CE4-BE91-6BDDFCDE7D8D}"/>
+    <hyperlink ref="L31" r:id="rId1" xr:uid="{4DDFA626-C1E3-4458-92A2-B7D165A0519C}"/>
+    <hyperlink ref="L7" r:id="rId2" xr:uid="{5ABDACB3-B3F4-4F86-99EC-4AA62FA84D21}"/>
+    <hyperlink ref="L17" r:id="rId3" xr:uid="{6459CE0B-A281-4375-9C7C-05121ADE6BE2}"/>
+    <hyperlink ref="L32" r:id="rId4" xr:uid="{018F4AFE-A58A-48E7-A5D8-D49BBBA7AF38}"/>
+    <hyperlink ref="L33" r:id="rId5" xr:uid="{84533807-29E2-4CAA-84C9-34900C15055C}"/>
+    <hyperlink ref="L35" r:id="rId6" xr:uid="{C14D6FD1-AEE2-4ECD-A527-6196769534BB}"/>
+    <hyperlink ref="L34" r:id="rId7" xr:uid="{1D36EC75-443F-4CE4-BE91-6BDDFCDE7D8D}"/>
+    <hyperlink ref="L4" r:id="rId8" xr:uid="{EA2BF17E-AEDD-418F-B946-1A51F7ADFB2B}"/>
+    <hyperlink ref="L30" r:id="rId9" xr:uid="{D1B46D99-B5EC-4C8E-9224-FE4D594B95AA}"/>
+    <hyperlink ref="L9" r:id="rId10" xr:uid="{0BF92FBB-E3CA-4ECC-840E-E24C686BC1A2}"/>
+    <hyperlink ref="L10" r:id="rId11" xr:uid="{760BC1CB-8B4B-441B-8268-FA0F281806D5}"/>
+    <hyperlink ref="L11" r:id="rId12" xr:uid="{530527DC-ED80-45C6-AB9A-5EA3FB072465}"/>
+    <hyperlink ref="L12" r:id="rId13" xr:uid="{7CAF7B79-8CAB-4E9D-AD8C-A7FE50B8F23A}"/>
+    <hyperlink ref="L13" r:id="rId14" xr:uid="{58E9F810-BF75-4A68-AAE9-F530F03DE5A6}"/>
+    <hyperlink ref="L14" r:id="rId15" xr:uid="{6BB873C0-FB4F-4330-BB12-175233D75E85}"/>
+    <hyperlink ref="L15" r:id="rId16" xr:uid="{C03B4D72-2A69-43BB-9CB2-3540A8576489}"/>
+    <hyperlink ref="L8" r:id="rId17" xr:uid="{419A9A14-A395-4481-B657-4D8207AD2077}"/>
+    <hyperlink ref="L18:L29" r:id="rId18" display="AliExpress" xr:uid="{3A0D5842-A681-46B6-B65F-70C433481904}"/>
+    <hyperlink ref="L18" r:id="rId19" xr:uid="{0C9AD063-EF43-48EE-B6D6-5A087B2D2756}"/>
+    <hyperlink ref="L19" r:id="rId20" xr:uid="{EE0CEFE6-9DCA-41E4-B625-3DA2B66AF10C}"/>
+    <hyperlink ref="L20" r:id="rId21" xr:uid="{922FB6AA-7CFB-45FA-96E3-C92762136D40}"/>
+    <hyperlink ref="L21" r:id="rId22" xr:uid="{4BDAA4AD-9A6F-443B-87ED-AE2AB83DBC61}"/>
+    <hyperlink ref="L22" r:id="rId23" xr:uid="{55BFF63F-1C91-4847-AA5F-A9ABF2839F31}"/>
+    <hyperlink ref="L23" r:id="rId24" xr:uid="{514B2E75-1B20-48E9-9CA0-76EF130FB9D3}"/>
+    <hyperlink ref="L24" r:id="rId25" xr:uid="{A0BEE243-3D46-4667-9B2B-52390856EBA5}"/>
+    <hyperlink ref="L25" r:id="rId26" xr:uid="{F7007339-A6F3-46FB-B47A-24C34A4B58ED}"/>
+    <hyperlink ref="L26" r:id="rId27" xr:uid="{84F3E837-CB20-4605-8A34-25AD337BB1E9}"/>
+    <hyperlink ref="L27" r:id="rId28" xr:uid="{5580C55D-C0BE-426D-BADE-687677D952FD}"/>
+    <hyperlink ref="L28" r:id="rId29" xr:uid="{0DA4CC6C-2226-45B9-B3BA-364C2DFD53EF}"/>
+    <hyperlink ref="L29" r:id="rId30" xr:uid="{7605B771-EC4A-4575-8456-9FE46D229D2F}"/>
+    <hyperlink ref="L16" r:id="rId31" xr:uid="{E588467F-8875-4F3D-BA7E-9367A9B8D12C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId32"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{882566EC-49D9-49EE-80AF-E86C05C8DBDB}">
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultColWidth="20.7109375" defaultRowHeight="24.95" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.7109375" style="3"/>
+    <col min="2" max="2" width="25.7109375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" style="3" customWidth="1"/>
+    <col min="4" max="5" width="20.7109375" style="3"/>
+    <col min="6" max="6" width="15.7109375" style="3" customWidth="1"/>
+    <col min="7" max="8" width="20.7109375" style="3"/>
+    <col min="9" max="9" width="10.7109375" style="3" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" style="3" customWidth="1"/>
+    <col min="11" max="16384" width="20.7109375" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="3"/>
+    </row>
+    <row r="2" spans="1:10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="3"/>
+    </row>
+    <row r="3" spans="1:10" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6">
+        <v>1.72</v>
+      </c>
+      <c r="E4" s="6">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="F4" s="9">
+        <v>1</v>
+      </c>
+      <c r="G4" s="6">
+        <f>Table1325[[#This Row],[Unit Price]]*Table1325[[#This Row],[Needed to Buy]]+Table1325[[#This Row],[Shipping]]</f>
+        <v>2.84</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" s="1">
+        <v>8</v>
+      </c>
+      <c r="D5" s="6">
+        <v>9.5299999999999994</v>
+      </c>
+      <c r="E5" s="6">
+        <v>5.94</v>
+      </c>
+      <c r="F5" s="9">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6">
+        <f>Table1325[[#This Row],[Unit Price]]*Table1325[[#This Row],[Needed to Buy]]+Table1325[[#This Row],[Shipping]]</f>
+        <v>15.469999999999999</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="1">
+        <v>12</v>
+      </c>
+      <c r="D6" s="6">
+        <v>31.45</v>
+      </c>
+      <c r="E6" s="6">
+        <v>2.81</v>
+      </c>
+      <c r="F6" s="9">
+        <v>1</v>
+      </c>
+      <c r="G6" s="6">
+        <f>Table1325[[#This Row],[Unit Price]]*Table1325[[#This Row],[Needed to Buy]]+Table1325[[#This Row],[Shipping]]</f>
+        <v>34.26</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="1">
+        <v>5</v>
+      </c>
+      <c r="D7" s="6">
+        <v>19.5</v>
+      </c>
+      <c r="E7" s="6">
+        <v>1.66</v>
+      </c>
+      <c r="F7" s="9">
+        <v>1</v>
+      </c>
+      <c r="G7" s="6">
+        <f>Table1325[[#This Row],[Unit Price]]*Table1325[[#This Row],[Needed to Buy]]+Table1325[[#This Row],[Shipping]]</f>
+        <v>21.16</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" s="1">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6">
+        <v>0</v>
+      </c>
+      <c r="E8" s="6">
+        <v>0</v>
+      </c>
+      <c r="F8" s="9">
+        <v>1</v>
+      </c>
+      <c r="G8" s="6">
+        <f>Table1325[[#This Row],[Unit Price]]*Table1325[[#This Row],[Needed to Buy]]+Table1325[[#This Row],[Shipping]]</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" s="4"/>
+    </row>
+    <row r="9" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="8">
+        <f>SUM(Table1325[Total Price])</f>
+        <v>73.72999999999999</v>
+      </c>
+      <c r="H9" s="8"/>
+      <c r="I9" s="5"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:I2"/>
+  </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="I4" r:id="rId1" xr:uid="{8A561FCD-3E62-4326-AC8C-BA6F7DA8F968}"/>
+    <hyperlink ref="I5" r:id="rId2" xr:uid="{4EEF68E0-6BE1-4A49-A727-CB71B6A61A5C}"/>
+    <hyperlink ref="I6" r:id="rId3" xr:uid="{FEE499EA-0091-42D0-88E0-7DCF10BB4B63}"/>
+    <hyperlink ref="I7" r:id="rId4" xr:uid="{63606D5D-FCBC-4DDF-A88A-CE7D04B70A8D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId5"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6197D644-F07B-4B07-BA89-84498DA20E66}">
   <dimension ref="A1:L19"/>
   <sheetFormatPr defaultColWidth="20.7109375" defaultRowHeight="24.95" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1784,37 +3293,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
       <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:12" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14" t="s">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
       <c r="L2" s="3"/>
     </row>
     <row r="3" spans="1:12" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2394,7 +3903,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8CFA2BC-95D1-4BFC-A97F-478F653543E5}">
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultColWidth="20.7109375" defaultRowHeight="24.95" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2403,35 +3912,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
       <c r="K1" s="3"/>
     </row>
     <row r="2" spans="1:11" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14" t="s">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
       <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:11" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>